<commit_message>
task132: realism rebuild after the leak reader (names, crews, service windows, cancellations, inspections, scopes, containers), world seed 147, answer 17 lots
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task132/golden/vpr340_psu_final_buy.xlsx
+++ b/task132/golden/vpr340_psu_final_buy.xlsx
@@ -2,7 +2,6 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
@@ -15,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -511,7 +510,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5">
@@ -521,7 +520,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>475</v>
+        <v>425</v>
       </c>
     </row>
     <row r="6">
@@ -531,7 +530,7 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>933375</v>
+        <v>835125</v>
       </c>
     </row>
     <row r="7">
@@ -541,7 +540,7 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>467.8</v>
+        <v>407.5</v>
       </c>
     </row>
     <row r="8">
@@ -551,7 +550,7 @@
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>39</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9">
@@ -561,7 +560,7 @@
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>98.3</v>
+        <v>98.90000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -620,19 +619,19 @@
     </row>
     <row r="2">
       <c r="A2" s="11" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B2" s="12" t="n">
-        <v>375</v>
+        <v>325</v>
       </c>
       <c r="C2" s="12" t="n">
-        <v>414</v>
+        <v>354</v>
       </c>
       <c r="D2" s="13" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="E2" s="14" t="n">
-        <v>736875</v>
+        <v>638625</v>
       </c>
       <c r="F2" s="15" t="inlineStr">
         <is>
@@ -642,19 +641,19 @@
     </row>
     <row r="3">
       <c r="A3" s="11" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B3" s="12" t="n">
-        <v>400</v>
+        <v>350</v>
       </c>
       <c r="C3" s="12" t="n">
-        <v>439</v>
+        <v>379</v>
       </c>
       <c r="D3" s="13" t="n">
-        <v>9.4</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="E3" s="14" t="n">
-        <v>786000</v>
+        <v>687750</v>
       </c>
       <c r="F3" s="15" t="inlineStr">
         <is>
@@ -664,19 +663,19 @@
     </row>
     <row r="4">
       <c r="A4" s="11" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B4" s="12" t="n">
-        <v>425</v>
+        <v>375</v>
       </c>
       <c r="C4" s="12" t="n">
-        <v>464</v>
+        <v>404</v>
       </c>
       <c r="D4" s="13" t="n">
-        <v>44.2</v>
+        <v>44.5</v>
       </c>
       <c r="E4" s="14" t="n">
-        <v>835125</v>
+        <v>736875</v>
       </c>
       <c r="F4" s="15" t="inlineStr">
         <is>
@@ -686,19 +685,19 @@
     </row>
     <row r="5">
       <c r="A5" s="11" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B5" s="12" t="n">
-        <v>450</v>
+        <v>400</v>
       </c>
       <c r="C5" s="12" t="n">
-        <v>489</v>
+        <v>429</v>
       </c>
       <c r="D5" s="13" t="n">
-        <v>84.2</v>
+        <v>86.2</v>
       </c>
       <c r="E5" s="14" t="n">
-        <v>884250</v>
+        <v>786000</v>
       </c>
       <c r="F5" s="15" t="inlineStr">
         <is>
@@ -708,19 +707,19 @@
     </row>
     <row r="6">
       <c r="A6" s="16" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B6" s="17" t="n">
-        <v>475</v>
+        <v>425</v>
       </c>
       <c r="C6" s="17" t="n">
-        <v>514</v>
+        <v>454</v>
       </c>
       <c r="D6" s="18" t="n">
-        <v>98.3</v>
+        <v>98.90000000000001</v>
       </c>
       <c r="E6" s="19" t="n">
-        <v>933375</v>
+        <v>835125</v>
       </c>
       <c r="F6" s="20" t="inlineStr">
         <is>
@@ -730,19 +729,19 @@
     </row>
     <row r="7">
       <c r="A7" s="11" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B7" s="12" t="n">
-        <v>500</v>
+        <v>450</v>
       </c>
       <c r="C7" s="12" t="n">
-        <v>539</v>
+        <v>479</v>
       </c>
       <c r="D7" s="13" t="n">
-        <v>99.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="E7" s="14" t="n">
-        <v>982500</v>
+        <v>884250</v>
       </c>
       <c r="F7" s="15" t="inlineStr">
         <is>
@@ -752,19 +751,19 @@
     </row>
     <row r="8">
       <c r="A8" s="11" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B8" s="12" t="n">
-        <v>525</v>
+        <v>475</v>
       </c>
       <c r="C8" s="12" t="n">
-        <v>564</v>
+        <v>504</v>
       </c>
       <c r="D8" s="13" t="n">
         <v>100</v>
       </c>
       <c r="E8" s="14" t="n">
-        <v>1031625</v>
+        <v>933375</v>
       </c>
       <c r="F8" s="15" t="inlineStr">
         <is>
@@ -815,7 +814,7 @@
         </is>
       </c>
       <c r="B2" s="13" t="n">
-        <v>17.2</v>
+        <v>16.6</v>
       </c>
     </row>
     <row r="3">
@@ -823,10 +822,10 @@
         <v>2027</v>
       </c>
       <c r="B3" s="13" t="n">
-        <v>68.2</v>
+        <v>63.7</v>
       </c>
       <c r="C3" s="12" t="n">
-        <v>1171</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="4">
@@ -834,10 +833,10 @@
         <v>2028</v>
       </c>
       <c r="B4" s="13" t="n">
-        <v>68.7</v>
+        <v>63.2</v>
       </c>
       <c r="C4" s="12" t="n">
-        <v>1052</v>
+        <v>1047</v>
       </c>
     </row>
     <row r="5">
@@ -845,10 +844,10 @@
         <v>2029</v>
       </c>
       <c r="B5" s="13" t="n">
-        <v>68.5</v>
+        <v>57.9</v>
       </c>
       <c r="C5" s="12" t="n">
-        <v>926</v>
+        <v>927</v>
       </c>
     </row>
     <row r="6">
@@ -856,10 +855,10 @@
         <v>2030</v>
       </c>
       <c r="B6" s="13" t="n">
-        <v>61.9</v>
+        <v>51.7</v>
       </c>
       <c r="C6" s="12" t="n">
-        <v>800</v>
+        <v>802</v>
       </c>
     </row>
     <row r="7">
@@ -867,10 +866,10 @@
         <v>2031</v>
       </c>
       <c r="B7" s="13" t="n">
-        <v>59.3</v>
+        <v>47.6</v>
       </c>
       <c r="C7" s="12" t="n">
-        <v>692</v>
+        <v>678</v>
       </c>
     </row>
     <row r="8">
@@ -878,10 +877,10 @@
         <v>2032</v>
       </c>
       <c r="B8" s="13" t="n">
-        <v>50.6</v>
+        <v>40.8</v>
       </c>
       <c r="C8" s="12" t="n">
-        <v>571</v>
+        <v>545</v>
       </c>
     </row>
     <row r="9">
@@ -889,10 +888,10 @@
         <v>2033</v>
       </c>
       <c r="B9" s="13" t="n">
-        <v>39.7</v>
+        <v>29.7</v>
       </c>
       <c r="C9" s="12" t="n">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="10">
@@ -900,10 +899,10 @@
         <v>2034</v>
       </c>
       <c r="B10" s="13" t="n">
-        <v>23.5</v>
+        <v>22</v>
       </c>
       <c r="C10" s="12" t="n">
-        <v>321</v>
+        <v>318</v>
       </c>
     </row>
     <row r="11">
@@ -911,10 +910,10 @@
         <v>2035</v>
       </c>
       <c r="B11" s="13" t="n">
-        <v>10.2</v>
+        <v>14.2</v>
       </c>
       <c r="C11" s="12" t="n">
-        <v>208</v>
+        <v>201</v>
       </c>
     </row>
     <row r="12">
@@ -924,7 +923,7 @@
         </is>
       </c>
       <c r="B12" s="18" t="n">
-        <v>467.8</v>
+        <v>407.5</v>
       </c>
     </row>
   </sheetData>
@@ -964,7 +963,7 @@
         </is>
       </c>
       <c r="B2" s="13" t="n">
-        <v>230.5</v>
+        <v>176.3</v>
       </c>
     </row>
     <row r="3">
@@ -974,7 +973,7 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>105.3</v>
+        <v>104.5</v>
       </c>
     </row>
     <row r="4">
@@ -984,7 +983,7 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>132</v>
+        <v>126.6</v>
       </c>
     </row>
   </sheetData>
@@ -1042,16 +1041,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C2" s="21" t="n">
-        <v>1564</v>
+        <v>1483.1</v>
       </c>
       <c r="D2" s="22" t="n">
-        <v>0.0026</v>
+        <v>0.004</v>
       </c>
       <c r="E2" s="21" t="n">
-        <v>124.2</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3">
@@ -1061,16 +1060,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C3" s="21" t="n">
-        <v>1770.8</v>
+        <v>1961.8</v>
       </c>
       <c r="D3" s="22" t="n">
-        <v>0.0124</v>
+        <v>0.0122</v>
       </c>
       <c r="E3" s="21" t="n">
-        <v>1047.2</v>
+        <v>1037.2</v>
       </c>
     </row>
     <row r="4">
@@ -1080,16 +1079,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C4" s="21" t="n">
-        <v>1671.8</v>
+        <v>1601.5</v>
       </c>
       <c r="D4" s="22" t="n">
         <v>0.0287</v>
       </c>
       <c r="E4" s="21" t="n">
-        <v>1655.2</v>
+        <v>1845</v>
       </c>
     </row>
     <row r="5">
@@ -1099,16 +1098,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="C5" s="21" t="n">
-        <v>1303.2</v>
+        <v>1052.8</v>
       </c>
       <c r="D5" s="22" t="n">
-        <v>0.066</v>
+        <v>0.0741</v>
       </c>
       <c r="E5" s="21" t="n">
-        <v>1543.2</v>
+        <v>1472.4</v>
       </c>
     </row>
     <row r="6">
@@ -1118,16 +1117,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="C6" s="21" t="n">
-        <v>504.1</v>
+        <v>585.1</v>
       </c>
       <c r="D6" s="22" t="n">
-        <v>0.1329</v>
+        <v>0.1538</v>
       </c>
       <c r="E6" s="21" t="n">
-        <v>1025.7</v>
+        <v>769.2</v>
       </c>
     </row>
     <row r="7">
@@ -1137,16 +1136,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C7" s="21" t="n">
-        <v>140.2</v>
+        <v>247.5</v>
       </c>
       <c r="D7" s="22" t="n">
-        <v>0.2782</v>
+        <v>0.1616</v>
       </c>
       <c r="E7" s="21" t="n">
-        <v>606.8</v>
+        <v>705.1</v>
       </c>
     </row>
   </sheetData>
@@ -1197,7 +1196,7 @@
     <row r="5">
       <c r="A5" s="23" t="inlineStr">
         <is>
-          <t>Available modules: 36 serviceable at Central Stores, North and South depots plus 3 at Veldtek under open RMA; 7 quarantined modules excluded (5).</t>
+          <t>Available modules: 23 serviceable at Central Stores, North and South depots plus 6 at Veldtek under open RMA; 7 quarantined modules excluded (5).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
task132 hardening loop 1: PSU wear-out by module age with replacement, staged programme, realism rebuild; answer 13 lots
Solver round 1 (both landed 17 lots by clipping exposure to the go-live window) sent the build
back to design. Loop 1 makes the replacement of failed modules the decisive forecast step,
adds the rotating-item history, the 2015 service-bulletin swaps, staged schemes by bay, and the
second leak read's realism fixes. Checks 65 pass, verifier pass, builds byte-identical.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task132/golden/vpr340_psu_final_buy.xlsx
+++ b/task132/golden/vpr340_psu_final_buy.xlsx
@@ -16,6 +16,140 @@
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="43">
+  <si>
+    <t>VPR-340 power supply module (VPR340-PSU-02): last-time buy</t>
+  </si>
+  <si>
+    <t>P&amp;C Asset Planning, prepared 7 October 2026 for the Director, Asset Management. Sized under AM-PC-014 rev 4.</t>
+  </si>
+  <si>
+    <t>Lots to order (25 modules per lot)</t>
+  </si>
+  <si>
+    <t>Modules to order</t>
+  </si>
+  <si>
+    <t>Cost at the last-time-buy price (CAD)</t>
+  </si>
+  <si>
+    <t>Expected failures, 1 Oct 2026 to end of support</t>
+  </si>
+  <si>
+    <t>Available modules at the 30 Sep 2026 count (serviceable plus at Veldtek repair)</t>
+  </si>
+  <si>
+    <t>Probability the stock covers every failure to end of support</t>
+  </si>
+  <si>
+    <t>Lots ordered</t>
+  </si>
+  <si>
+    <t>Modules ordered</t>
+  </si>
+  <si>
+    <t>Modules available with the buy</t>
+  </si>
+  <si>
+    <t>Cover probability (%)</t>
+  </si>
+  <si>
+    <t>Cost (CAD)</t>
+  </si>
+  <si>
+    <t>Meets 95%</t>
+  </si>
+  <si>
+    <t>no</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>Expected PSU failures</t>
+  </si>
+  <si>
+    <t>Relays supported on 1 January</t>
+  </si>
+  <si>
+    <t>2026 (Oct-Dec)</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Operating region (from April 2024)</t>
+  </si>
+  <si>
+    <t>Expected PSU failures to end of support</t>
+  </si>
+  <si>
+    <t>North</t>
+  </si>
+  <si>
+    <t>Central</t>
+  </si>
+  <si>
+    <t>South</t>
+  </si>
+  <si>
+    <t>Module age band (years)</t>
+  </si>
+  <si>
+    <t>PSU failures Jan 2021 to Sep 2026</t>
+  </si>
+  <si>
+    <t>Module-years in service Jan 2021 to Sep 2026</t>
+  </si>
+  <si>
+    <t>Failures per module-year</t>
+  </si>
+  <si>
+    <t>Expected module-years to end of support</t>
+  </si>
+  <si>
+    <t>Expected failures</t>
+  </si>
+  <si>
+    <t>0-9</t>
+  </si>
+  <si>
+    <t>10-14</t>
+  </si>
+  <si>
+    <t>15-19</t>
+  </si>
+  <si>
+    <t>20-24</t>
+  </si>
+  <si>
+    <t>25+</t>
+  </si>
+  <si>
+    <t>Failures: corrective (CM, EM) work orders on VPR-340 relays with failed component PSU, status COMP or CLOSE (AM-PC-014 5.1). Each failure takes the age of the module it removed, from that module's fitted date in the rotating-item history (5.2).</t>
+  </si>
+  <si>
+    <t>Rates: module-years are counted from the January 2021 go-live, when the work-order history begins; a module fitted earlier enters the count at go-live at the age it had then (5.3).</t>
+  </si>
+  <si>
+    <t>Expected module-years: each supported relay's present module is aged month by month. A module that fails is replaced from stock by a new module, which counts in the 0-9 band from the following month, so each month's module-years are split between the present module (by the chance it has not yet failed) and its replacement (6.1, 6.2).</t>
+  </si>
+  <si>
+    <t>Support ends in the commissioning month of the scheme, or the stage of a staged scheme, that replaces the relay's bay in the approved 2026 programme; relays at stations with no scheme in the period are supported to December 2035 (4.1, 4.2).</t>
+  </si>
+  <si>
+    <t>Available modules: 12 serviceable at Central Stores, North and South depots plus 2 at Veldtek under open RMA; 7 quarantined modules excluded (7).</t>
+  </si>
+  <si>
+    <t>Cover is the Poisson probability that available modules plus the buy meet all failures to end of support (8.1, 8.2).</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -77,44 +211,44 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="24">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" applyAlignment="1" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" applyAlignment="1" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" applyAlignment="1" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -490,77 +624,61 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>VPR-340 power supply module (VPR340-PSU-02): last-time buy</t>
-        </is>
+      <c r="A1" s="1" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>P&amp;C Asset Planning, prepared 7 October 2026 for the Director, Asset Management. Sized under AM-PC-014 rev 3.</t>
-        </is>
+      <c r="A2" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Lots to order (25 modules per lot)</t>
-        </is>
+      <c r="A4" s="3" t="s">
+        <v>2</v>
       </c>
       <c r="B4" s="4" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Modules to order</t>
-        </is>
+      <c r="A5" t="s">
+        <v>3</v>
       </c>
       <c r="B5" s="5" t="n">
-        <v>425</v>
+        <v>325</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Cost at the last-time-buy price (CAD)</t>
-        </is>
+      <c r="A6" t="s">
+        <v>4</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>835125</v>
+        <v>638625</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Expected failures, 1 Oct 2026 to end of support</t>
-        </is>
+      <c r="A7" t="s">
+        <v>5</v>
       </c>
       <c r="B7" s="7" t="n">
-        <v>407.5</v>
+        <v>297.9</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Available modules at the 30 Sep 2026 count (serviceable plus at Veldtek repair)</t>
-        </is>
+      <c r="A8" t="s">
+        <v>6</v>
       </c>
       <c r="B8" s="8" t="n">
-        <v>29</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Probability the stock covers every failure to end of support</t>
-        </is>
+      <c r="A9" t="s">
+        <v>7</v>
       </c>
       <c r="B9" s="9" t="n">
-        <v>98.90000000000001</v>
+        <v>99.09999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -574,7 +692,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -586,189 +704,323 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
-        <is>
-          <t>Lots ordered</t>
-        </is>
-      </c>
-      <c r="B1" s="10" t="inlineStr">
-        <is>
-          <t>Modules ordered</t>
-        </is>
-      </c>
-      <c r="C1" s="10" t="inlineStr">
-        <is>
-          <t>Modules available with the buy</t>
-        </is>
-      </c>
-      <c r="D1" s="10" t="inlineStr">
-        <is>
-          <t>Cover probability (%)</t>
-        </is>
-      </c>
-      <c r="E1" s="10" t="inlineStr">
-        <is>
-          <t>Cost (CAD)</t>
-        </is>
-      </c>
-      <c r="F1" s="10" t="inlineStr">
-        <is>
-          <t>Meets 95%</t>
-        </is>
+      <c r="A1" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="11" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B2" s="12" t="n">
-        <v>325</v>
+        <v>200</v>
       </c>
       <c r="C2" s="12" t="n">
-        <v>354</v>
+        <v>214</v>
       </c>
       <c r="D2" s="13" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="E2" s="14" t="n">
-        <v>638625</v>
-      </c>
-      <c r="F2" s="15" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
+        <v>393000</v>
+      </c>
+      <c r="F2" s="15" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="11" t="n">
+        <v>9</v>
+      </c>
+      <c r="B3" s="12" t="n">
+        <v>225</v>
+      </c>
+      <c r="C3" s="12" t="n">
+        <v>239</v>
+      </c>
+      <c r="D3" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="14" t="n">
+        <v>442125</v>
+      </c>
+      <c r="F3" s="15" t="s">
         <v>14</v>
-      </c>
-      <c r="B3" s="12" t="n">
-        <v>350</v>
-      </c>
-      <c r="C3" s="12" t="n">
-        <v>379</v>
-      </c>
-      <c r="D3" s="13" t="n">
-        <v>8.199999999999999</v>
-      </c>
-      <c r="E3" s="14" t="n">
-        <v>687750</v>
-      </c>
-      <c r="F3" s="15" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="B4" s="12" t="n">
-        <v>375</v>
+        <v>250</v>
       </c>
       <c r="C4" s="12" t="n">
-        <v>404</v>
+        <v>264</v>
       </c>
       <c r="D4" s="13" t="n">
-        <v>44.5</v>
+        <v>2.5</v>
       </c>
       <c r="E4" s="14" t="n">
-        <v>736875</v>
-      </c>
-      <c r="F4" s="15" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
+        <v>491250</v>
+      </c>
+      <c r="F4" s="15" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B5" s="12" t="n">
-        <v>400</v>
+        <v>275</v>
       </c>
       <c r="C5" s="12" t="n">
-        <v>429</v>
+        <v>289</v>
       </c>
       <c r="D5" s="13" t="n">
-        <v>86.2</v>
+        <v>31.6</v>
       </c>
       <c r="E5" s="14" t="n">
-        <v>786000</v>
-      </c>
-      <c r="F5" s="15" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
+        <v>540375</v>
+      </c>
+      <c r="F5" s="15" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="n">
-        <v>17</v>
-      </c>
-      <c r="B6" s="17" t="n">
-        <v>425</v>
-      </c>
-      <c r="C6" s="17" t="n">
-        <v>454</v>
-      </c>
-      <c r="D6" s="18" t="n">
-        <v>98.90000000000001</v>
-      </c>
-      <c r="E6" s="19" t="n">
-        <v>835125</v>
-      </c>
-      <c r="F6" s="20" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
+      <c r="A6" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="B6" s="12" t="n">
+        <v>300</v>
+      </c>
+      <c r="C6" s="12" t="n">
+        <v>314</v>
+      </c>
+      <c r="D6" s="13" t="n">
+        <v>83.2</v>
+      </c>
+      <c r="E6" s="14" t="n">
+        <v>589500</v>
+      </c>
+      <c r="F6" s="15" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="n">
-        <v>18</v>
-      </c>
-      <c r="B7" s="12" t="n">
-        <v>450</v>
-      </c>
-      <c r="C7" s="12" t="n">
-        <v>479</v>
-      </c>
-      <c r="D7" s="13" t="n">
-        <v>100</v>
-      </c>
-      <c r="E7" s="14" t="n">
-        <v>884250</v>
-      </c>
-      <c r="F7" s="15" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
+      <c r="A7" s="16" t="n">
+        <v>13</v>
+      </c>
+      <c r="B7" s="17" t="n">
+        <v>325</v>
+      </c>
+      <c r="C7" s="17" t="n">
+        <v>339</v>
+      </c>
+      <c r="D7" s="18" t="n">
+        <v>99.09999999999999</v>
+      </c>
+      <c r="E7" s="19" t="n">
+        <v>638625</v>
+      </c>
+      <c r="F7" s="20" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="B8" s="12" t="n">
-        <v>475</v>
+        <v>350</v>
       </c>
       <c r="C8" s="12" t="n">
-        <v>504</v>
+        <v>364</v>
       </c>
       <c r="D8" s="13" t="n">
         <v>100</v>
       </c>
       <c r="E8" s="14" t="n">
+        <v>687750</v>
+      </c>
+      <c r="F8" s="15" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="n">
+        <v>15</v>
+      </c>
+      <c r="B9" s="12" t="n">
+        <v>375</v>
+      </c>
+      <c r="C9" s="12" t="n">
+        <v>389</v>
+      </c>
+      <c r="D9" s="13" t="n">
+        <v>100</v>
+      </c>
+      <c r="E9" s="14" t="n">
+        <v>736875</v>
+      </c>
+      <c r="F9" s="15" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="n">
+        <v>16</v>
+      </c>
+      <c r="B10" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="C10" s="12" t="n">
+        <v>414</v>
+      </c>
+      <c r="D10" s="13" t="n">
+        <v>100</v>
+      </c>
+      <c r="E10" s="14" t="n">
+        <v>786000</v>
+      </c>
+      <c r="F10" s="15" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="n">
+        <v>17</v>
+      </c>
+      <c r="B11" s="12" t="n">
+        <v>425</v>
+      </c>
+      <c r="C11" s="12" t="n">
+        <v>439</v>
+      </c>
+      <c r="D11" s="13" t="n">
+        <v>100</v>
+      </c>
+      <c r="E11" s="14" t="n">
+        <v>835125</v>
+      </c>
+      <c r="F11" s="15" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="n">
+        <v>18</v>
+      </c>
+      <c r="B12" s="12" t="n">
+        <v>450</v>
+      </c>
+      <c r="C12" s="12" t="n">
+        <v>464</v>
+      </c>
+      <c r="D12" s="13" t="n">
+        <v>100</v>
+      </c>
+      <c r="E12" s="14" t="n">
+        <v>884250</v>
+      </c>
+      <c r="F12" s="15" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="n">
+        <v>19</v>
+      </c>
+      <c r="B13" s="12" t="n">
+        <v>475</v>
+      </c>
+      <c r="C13" s="12" t="n">
+        <v>489</v>
+      </c>
+      <c r="D13" s="13" t="n">
+        <v>100</v>
+      </c>
+      <c r="E13" s="14" t="n">
         <v>933375</v>
       </c>
-      <c r="F8" s="15" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
+      <c r="F13" s="15" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="B14" s="12" t="n">
+        <v>500</v>
+      </c>
+      <c r="C14" s="12" t="n">
+        <v>514</v>
+      </c>
+      <c r="D14" s="13" t="n">
+        <v>100</v>
+      </c>
+      <c r="E14" s="14" t="n">
+        <v>982500</v>
+      </c>
+      <c r="F14" s="15" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="n">
+        <v>21</v>
+      </c>
+      <c r="B15" s="12" t="n">
+        <v>525</v>
+      </c>
+      <c r="C15" s="12" t="n">
+        <v>539</v>
+      </c>
+      <c r="D15" s="13" t="n">
+        <v>100</v>
+      </c>
+      <c r="E15" s="14" t="n">
+        <v>1031625</v>
+      </c>
+      <c r="F15" s="15" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="n">
+        <v>22</v>
+      </c>
+      <c r="B16" s="12" t="n">
+        <v>550</v>
+      </c>
+      <c r="C16" s="12" t="n">
+        <v>564</v>
+      </c>
+      <c r="D16" s="13" t="n">
+        <v>100</v>
+      </c>
+      <c r="E16" s="14" t="n">
+        <v>1080750</v>
+      </c>
+      <c r="F16" s="15" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -791,30 +1043,22 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
-        <is>
-          <t>Year</t>
-        </is>
-      </c>
-      <c r="B1" s="10" t="inlineStr">
-        <is>
-          <t>Expected PSU failures</t>
-        </is>
-      </c>
-      <c r="C1" s="10" t="inlineStr">
-        <is>
-          <t>Relays supported on 1 January</t>
-        </is>
+      <c r="A1" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026 (Oct-Dec)</t>
-        </is>
+      <c r="A2" t="s">
+        <v>19</v>
       </c>
       <c r="B2" s="13" t="n">
-        <v>16.6</v>
+        <v>11.3</v>
       </c>
     </row>
     <row r="3">
@@ -822,10 +1066,10 @@
         <v>2027</v>
       </c>
       <c r="B3" s="13" t="n">
-        <v>63.7</v>
+        <v>45.4</v>
       </c>
       <c r="C3" s="12" t="n">
-        <v>1170</v>
+        <v>1162</v>
       </c>
     </row>
     <row r="4">
@@ -833,10 +1077,10 @@
         <v>2028</v>
       </c>
       <c r="B4" s="13" t="n">
-        <v>63.2</v>
+        <v>45</v>
       </c>
       <c r="C4" s="12" t="n">
-        <v>1047</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="5">
@@ -844,10 +1088,10 @@
         <v>2029</v>
       </c>
       <c r="B5" s="13" t="n">
-        <v>57.9</v>
+        <v>43.5</v>
       </c>
       <c r="C5" s="12" t="n">
-        <v>927</v>
+        <v>999</v>
       </c>
     </row>
     <row r="6">
@@ -855,10 +1099,10 @@
         <v>2030</v>
       </c>
       <c r="B6" s="13" t="n">
-        <v>51.7</v>
+        <v>40</v>
       </c>
       <c r="C6" s="12" t="n">
-        <v>802</v>
+        <v>909</v>
       </c>
     </row>
     <row r="7">
@@ -866,10 +1110,10 @@
         <v>2031</v>
       </c>
       <c r="B7" s="13" t="n">
-        <v>47.6</v>
+        <v>34.1</v>
       </c>
       <c r="C7" s="12" t="n">
-        <v>678</v>
+        <v>796</v>
       </c>
     </row>
     <row r="8">
@@ -877,10 +1121,10 @@
         <v>2032</v>
       </c>
       <c r="B8" s="13" t="n">
-        <v>40.8</v>
+        <v>29.4</v>
       </c>
       <c r="C8" s="12" t="n">
-        <v>545</v>
+        <v>669</v>
       </c>
     </row>
     <row r="9">
@@ -888,10 +1132,10 @@
         <v>2033</v>
       </c>
       <c r="B9" s="13" t="n">
-        <v>29.7</v>
+        <v>23.3</v>
       </c>
       <c r="C9" s="12" t="n">
-        <v>439</v>
+        <v>565</v>
       </c>
     </row>
     <row r="10">
@@ -899,10 +1143,10 @@
         <v>2034</v>
       </c>
       <c r="B10" s="13" t="n">
-        <v>22</v>
+        <v>16.9</v>
       </c>
       <c r="C10" s="12" t="n">
-        <v>318</v>
+        <v>381</v>
       </c>
     </row>
     <row r="11">
@@ -910,20 +1154,18 @@
         <v>2035</v>
       </c>
       <c r="B11" s="13" t="n">
-        <v>14.2</v>
+        <v>8.9</v>
       </c>
       <c r="C11" s="12" t="n">
-        <v>201</v>
+        <v>218</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
+      <c r="A12" s="3" t="s">
+        <v>20</v>
       </c>
       <c r="B12" s="18" t="n">
-        <v>407.5</v>
+        <v>297.9</v>
       </c>
     </row>
   </sheetData>
@@ -945,45 +1187,35 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
-        <is>
-          <t>Operating region (from April 2024)</t>
-        </is>
-      </c>
-      <c r="B1" s="10" t="inlineStr">
-        <is>
-          <t>Expected PSU failures to end of support</t>
-        </is>
+      <c r="A1" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>North</t>
-        </is>
+      <c r="A2" t="s">
+        <v>23</v>
       </c>
       <c r="B2" s="13" t="n">
-        <v>176.3</v>
+        <v>87.09999999999999</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Central</t>
-        </is>
+      <c r="A3" t="s">
+        <v>24</v>
       </c>
       <c r="B3" s="13" t="n">
-        <v>104.5</v>
+        <v>121.7</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>South</t>
-        </is>
+      <c r="A4" t="s">
+        <v>25</v>
       </c>
       <c r="B4" s="13" t="n">
-        <v>126.6</v>
+        <v>89.09999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -997,155 +1229,146 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
-        <is>
-          <t>Age band (years)</t>
-        </is>
-      </c>
-      <c r="B1" s="10" t="inlineStr">
-        <is>
-          <t>PSU failures Jan 2021 to Sep 2026</t>
-        </is>
-      </c>
-      <c r="C1" s="10" t="inlineStr">
-        <is>
-          <t>Relay-years in service Jan 2021 to Sep 2026</t>
-        </is>
-      </c>
-      <c r="D1" s="10" t="inlineStr">
-        <is>
-          <t>Failures per relay-year</t>
-        </is>
-      </c>
-      <c r="E1" s="10" t="inlineStr">
-        <is>
-          <t>Relay-years to end of support</t>
-        </is>
+      <c r="A1" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>0-9</t>
-        </is>
+      <c r="A2" t="s">
+        <v>32</v>
       </c>
       <c r="B2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C2" s="21" t="n">
-        <v>1483.1</v>
+        <v>2567.6</v>
       </c>
       <c r="D2" s="22" t="n">
-        <v>0.004</v>
+        <v>0.0019</v>
       </c>
       <c r="E2" s="21" t="n">
-        <v>107</v>
+        <v>2066</v>
+      </c>
+      <c r="F2" s="13" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>10-14</t>
-        </is>
+      <c r="A3" t="s">
+        <v>33</v>
       </c>
       <c r="B3" t="n">
-        <v>24</v>
+        <v>51</v>
       </c>
       <c r="C3" s="21" t="n">
-        <v>1961.8</v>
+        <v>2228.3</v>
       </c>
       <c r="D3" s="22" t="n">
-        <v>0.0122</v>
+        <v>0.0229</v>
       </c>
       <c r="E3" s="21" t="n">
-        <v>1037.2</v>
+        <v>1187.1</v>
+      </c>
+      <c r="F3" s="13" t="n">
+        <v>27.2</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>15-19</t>
-        </is>
+      <c r="A4" t="s">
+        <v>34</v>
       </c>
       <c r="B4" t="n">
-        <v>46</v>
+        <v>61</v>
       </c>
       <c r="C4" s="21" t="n">
-        <v>1601.5</v>
+        <v>1417.2</v>
       </c>
       <c r="D4" s="22" t="n">
-        <v>0.0287</v>
+        <v>0.043</v>
       </c>
       <c r="E4" s="21" t="n">
-        <v>1845</v>
+        <v>1838</v>
+      </c>
+      <c r="F4" s="13" t="n">
+        <v>79.09999999999999</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>20-24</t>
-        </is>
+      <c r="A5" t="s">
+        <v>35</v>
       </c>
       <c r="B5" t="n">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="C5" s="21" t="n">
-        <v>1052.8</v>
+        <v>662</v>
       </c>
       <c r="D5" s="22" t="n">
-        <v>0.0741</v>
+        <v>0.0997</v>
       </c>
       <c r="E5" s="21" t="n">
-        <v>1472.4</v>
+        <v>1141.5</v>
+      </c>
+      <c r="F5" s="13" t="n">
+        <v>113.8</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>25-29</t>
-        </is>
+      <c r="A6" t="s">
+        <v>36</v>
       </c>
       <c r="B6" t="n">
-        <v>90</v>
+        <v>14</v>
       </c>
       <c r="C6" s="21" t="n">
-        <v>585.1</v>
+        <v>56.5</v>
       </c>
       <c r="D6" s="22" t="n">
-        <v>0.1538</v>
+        <v>0.2478</v>
       </c>
       <c r="E6" s="21" t="n">
-        <v>769.2</v>
+        <v>297.7</v>
+      </c>
+      <c r="F6" s="13" t="n">
+        <v>73.8</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>30+</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>40</v>
-      </c>
-      <c r="C7" s="21" t="n">
-        <v>247.5</v>
-      </c>
-      <c r="D7" s="22" t="n">
-        <v>0.1616</v>
-      </c>
-      <c r="E7" s="21" t="n">
-        <v>705.1</v>
+      <c r="A7" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>197</v>
+      </c>
+      <c r="F7" s="18" t="n">
+        <v>297.9</v>
       </c>
     </row>
   </sheetData>
@@ -1166,45 +1389,33 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="23" t="inlineStr">
-        <is>
-          <t>Failures are corrective (CM, EM) work orders on VPR-340 relays with failed component PSU, status COMP or CLOSE (AM-PC-014 4.1).</t>
-        </is>
+      <c r="A1" s="23" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="23" t="inlineStr">
-        <is>
-          <t>The EAM work-order history starts at the 1 January 2021 go-live, so relay-years are counted from that date: a relay-year before 2021 has no work order that could record its failures.</t>
-        </is>
+      <c r="A2" s="23" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="23" t="inlineStr">
-        <is>
-          <t>Ages are completed years on the first of each month from the register's installation date; relays count for a month when in service on its first day (4.2, 4.3).</t>
-        </is>
+      <c r="A3" s="23" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="23" t="inlineStr">
-        <is>
-          <t>Support ends in the commissioning month of the substation's scheme in the approved 2026 programme; substations with no scheme are supported to December 2035 (3.1, 3.2).</t>
-        </is>
+      <c r="A4" s="23" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="inlineStr">
-        <is>
-          <t>Available modules: 23 serviceable at Central Stores, North and South depots plus 6 at Veldtek under open RMA; 7 quarantined modules excluded (5).</t>
-        </is>
+      <c r="A5" s="23" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="inlineStr">
-        <is>
-          <t>Cover is the Poisson probability that available modules plus the buy meet all failures to end of support (6.1, 6.2).</t>
-        </is>
+      <c r="A6" s="23" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
task132 loop 1: realism rebuild after the reader (16 findings: containers, working-day calendars, corrective work, cutovers, programme scope, RMA, reclosing, EOL terms), Tarrock rename; answer unchanged at 13 lots
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task132/golden/vpr340_psu_final_buy.xlsx
+++ b/task132/golden/vpr340_psu_final_buy.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <workbookPr defaultThemeVersion="166925"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E1A4429-1A48-47A3-B72C-345A18A5DECE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{AA6AA2A3-D398-41C7-A988-ABB893934BF3}"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buy" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lot settings" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outlook by year" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By region" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Failure rates" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Buy" sheetId="1" r:id="rId1"/>
+    <sheet name="Lot settings" sheetId="2" r:id="rId2"/>
+    <sheet name="Outlook by year" sheetId="3" r:id="rId3"/>
+    <sheet name="By region" sheetId="4" r:id="rId4"/>
+    <sheet name="Failure rates" sheetId="5" r:id="rId5"/>
+    <sheet name="Notes" sheetId="6" r:id="rId6"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
@@ -153,7 +154,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="5">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
@@ -161,40 +162,58 @@
     <numFmt numFmtId="167" formatCode="0.0"/>
     <numFmt numFmtId="168" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
       <sz val="13"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <i val="1"/>
-      <color rgb="005A6A72"/>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF5A6A72"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002F6B55"/>
+        <fgColor rgb="FF2F6B55"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -212,118 +231,51 @@
   </cellStyleXfs>
   <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" applyAlignment="1" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" xfId="0">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" xfId="0">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" applyAlignment="1" xfId="0">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" applyAlignment="1" xfId="0">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" xfId="0">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
 </styleSheet>
 </file>
 
@@ -338,44 +290,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1F497D"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="EEECE1"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4F81BD"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="C0504D"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9BBB59"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064A2"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4BACC6"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="F79646"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000FF"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="800080"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hans" typeface="等线 Light"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -404,12 +356,12 @@
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="游明朝"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hans" typeface="等线"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -611,99 +563,91 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB2EA079-D595-4AFD-B427-A93BB6070ED6}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col width="74" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col min="1" max="1" width="74.7109375" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="4">
         <v>13</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="5" t="n">
+      <c r="B5" s="5">
         <v>325</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="6" t="n">
+      <c r="B6" s="6">
         <v>638625</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="7" t="n">
+      <c r="B7" s="7">
         <v>297.9</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="8" t="n">
+      <c r="B8" s="8">
         <v>14</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="9" t="n">
+      <c r="B9" s="9">
         <v>99.09999999999999</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6045485-23FD-4FD8-8A29-09E4CE58DF5A}">
   <dimension ref="A1:F16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="2" width="15.7109375" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" customWidth="1"/>
+    <col min="4" max="4" width="16.7109375" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" customWidth="1"/>
+    <col min="6" max="6" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>8</v>
       </c>
@@ -723,300 +667,300 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="11" t="n">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="11">
         <v>8</v>
       </c>
-      <c r="B2" s="12" t="n">
+      <c r="B2" s="12">
         <v>200</v>
       </c>
-      <c r="C2" s="12" t="n">
+      <c r="C2" s="12">
         <v>214</v>
       </c>
-      <c r="D2" s="13" t="n">
+      <c r="D2" s="13">
         <v>0</v>
       </c>
-      <c r="E2" s="14" t="n">
+      <c r="E2" s="14">
         <v>393000</v>
       </c>
       <c r="F2" s="15" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="11" t="n">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="11">
         <v>9</v>
       </c>
-      <c r="B3" s="12" t="n">
+      <c r="B3" s="12">
         <v>225</v>
       </c>
-      <c r="C3" s="12" t="n">
+      <c r="C3" s="12">
         <v>239</v>
       </c>
-      <c r="D3" s="13" t="n">
+      <c r="D3" s="13">
         <v>0</v>
       </c>
-      <c r="E3" s="14" t="n">
+      <c r="E3" s="14">
         <v>442125</v>
       </c>
       <c r="F3" s="15" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="11" t="n">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="11">
         <v>10</v>
       </c>
-      <c r="B4" s="12" t="n">
+      <c r="B4" s="12">
         <v>250</v>
       </c>
-      <c r="C4" s="12" t="n">
+      <c r="C4" s="12">
         <v>264</v>
       </c>
-      <c r="D4" s="13" t="n">
+      <c r="D4" s="13">
         <v>2.5</v>
       </c>
-      <c r="E4" s="14" t="n">
+      <c r="E4" s="14">
         <v>491250</v>
       </c>
       <c r="F4" s="15" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="11" t="n">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="11">
         <v>11</v>
       </c>
-      <c r="B5" s="12" t="n">
+      <c r="B5" s="12">
         <v>275</v>
       </c>
-      <c r="C5" s="12" t="n">
+      <c r="C5" s="12">
         <v>289</v>
       </c>
-      <c r="D5" s="13" t="n">
+      <c r="D5" s="13">
         <v>31.6</v>
       </c>
-      <c r="E5" s="14" t="n">
+      <c r="E5" s="14">
         <v>540375</v>
       </c>
       <c r="F5" s="15" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="11" t="n">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="11">
         <v>12</v>
       </c>
-      <c r="B6" s="12" t="n">
+      <c r="B6" s="12">
         <v>300</v>
       </c>
-      <c r="C6" s="12" t="n">
+      <c r="C6" s="12">
         <v>314</v>
       </c>
-      <c r="D6" s="13" t="n">
+      <c r="D6" s="13">
         <v>83.2</v>
       </c>
-      <c r="E6" s="14" t="n">
+      <c r="E6" s="14">
         <v>589500</v>
       </c>
       <c r="F6" s="15" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="16" t="n">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="16">
         <v>13</v>
       </c>
-      <c r="B7" s="17" t="n">
+      <c r="B7" s="17">
         <v>325</v>
       </c>
-      <c r="C7" s="17" t="n">
+      <c r="C7" s="17">
         <v>339</v>
       </c>
-      <c r="D7" s="18" t="n">
+      <c r="D7" s="18">
         <v>99.09999999999999</v>
       </c>
-      <c r="E7" s="19" t="n">
+      <c r="E7" s="19">
         <v>638625</v>
       </c>
       <c r="F7" s="20" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="11" t="n">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="11">
         <v>14</v>
       </c>
-      <c r="B8" s="12" t="n">
+      <c r="B8" s="12">
         <v>350</v>
       </c>
-      <c r="C8" s="12" t="n">
+      <c r="C8" s="12">
         <v>364</v>
       </c>
-      <c r="D8" s="13" t="n">
+      <c r="D8" s="13">
         <v>100</v>
       </c>
-      <c r="E8" s="14" t="n">
+      <c r="E8" s="14">
         <v>687750</v>
       </c>
       <c r="F8" s="15" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="11" t="n">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="11">
         <v>15</v>
       </c>
-      <c r="B9" s="12" t="n">
+      <c r="B9" s="12">
         <v>375</v>
       </c>
-      <c r="C9" s="12" t="n">
+      <c r="C9" s="12">
         <v>389</v>
       </c>
-      <c r="D9" s="13" t="n">
+      <c r="D9" s="13">
         <v>100</v>
       </c>
-      <c r="E9" s="14" t="n">
+      <c r="E9" s="14">
         <v>736875</v>
       </c>
       <c r="F9" s="15" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="11" t="n">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="11">
         <v>16</v>
       </c>
-      <c r="B10" s="12" t="n">
+      <c r="B10" s="12">
         <v>400</v>
       </c>
-      <c r="C10" s="12" t="n">
+      <c r="C10" s="12">
         <v>414</v>
       </c>
-      <c r="D10" s="13" t="n">
+      <c r="D10" s="13">
         <v>100</v>
       </c>
-      <c r="E10" s="14" t="n">
+      <c r="E10" s="14">
         <v>786000</v>
       </c>
       <c r="F10" s="15" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="11" t="n">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="11">
         <v>17</v>
       </c>
-      <c r="B11" s="12" t="n">
+      <c r="B11" s="12">
         <v>425</v>
       </c>
-      <c r="C11" s="12" t="n">
+      <c r="C11" s="12">
         <v>439</v>
       </c>
-      <c r="D11" s="13" t="n">
+      <c r="D11" s="13">
         <v>100</v>
       </c>
-      <c r="E11" s="14" t="n">
+      <c r="E11" s="14">
         <v>835125</v>
       </c>
       <c r="F11" s="15" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="11" t="n">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="11">
         <v>18</v>
       </c>
-      <c r="B12" s="12" t="n">
+      <c r="B12" s="12">
         <v>450</v>
       </c>
-      <c r="C12" s="12" t="n">
+      <c r="C12" s="12">
         <v>464</v>
       </c>
-      <c r="D12" s="13" t="n">
+      <c r="D12" s="13">
         <v>100</v>
       </c>
-      <c r="E12" s="14" t="n">
+      <c r="E12" s="14">
         <v>884250</v>
       </c>
       <c r="F12" s="15" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="11" t="n">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="11">
         <v>19</v>
       </c>
-      <c r="B13" s="12" t="n">
+      <c r="B13" s="12">
         <v>475</v>
       </c>
-      <c r="C13" s="12" t="n">
+      <c r="C13" s="12">
         <v>489</v>
       </c>
-      <c r="D13" s="13" t="n">
+      <c r="D13" s="13">
         <v>100</v>
       </c>
-      <c r="E13" s="14" t="n">
+      <c r="E13" s="14">
         <v>933375</v>
       </c>
       <c r="F13" s="15" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="11" t="n">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="11">
         <v>20</v>
       </c>
-      <c r="B14" s="12" t="n">
+      <c r="B14" s="12">
         <v>500</v>
       </c>
-      <c r="C14" s="12" t="n">
+      <c r="C14" s="12">
         <v>514</v>
       </c>
-      <c r="D14" s="13" t="n">
+      <c r="D14" s="13">
         <v>100</v>
       </c>
-      <c r="E14" s="14" t="n">
+      <c r="E14" s="14">
         <v>982500</v>
       </c>
       <c r="F14" s="15" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="11" t="n">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="11">
         <v>21</v>
       </c>
-      <c r="B15" s="12" t="n">
+      <c r="B15" s="12">
         <v>525</v>
       </c>
-      <c r="C15" s="12" t="n">
+      <c r="C15" s="12">
         <v>539</v>
       </c>
-      <c r="D15" s="13" t="n">
+      <c r="D15" s="13">
         <v>100</v>
       </c>
-      <c r="E15" s="14" t="n">
+      <c r="E15" s="14">
         <v>1031625</v>
       </c>
       <c r="F15" s="15" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="11" t="n">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="11">
         <v>22</v>
       </c>
-      <c r="B16" s="12" t="n">
+      <c r="B16" s="12">
         <v>550</v>
       </c>
-      <c r="C16" s="12" t="n">
+      <c r="C16" s="12">
         <v>564</v>
       </c>
-      <c r="D16" s="13" t="n">
+      <c r="D16" s="13">
         <v>100</v>
       </c>
-      <c r="E16" s="14" t="n">
+      <c r="E16" s="14">
         <v>1080750</v>
       </c>
       <c r="F16" s="15" t="s">
@@ -1024,25 +968,21 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{936C42E8-E7BF-4BEB-8BCE-97E31CB10092}">
   <dimension ref="A1:C12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col min="1" max="1" width="14.7109375" customWidth="1"/>
+    <col min="2" max="2" width="20.7109375" customWidth="1"/>
+    <col min="3" max="3" width="22.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>16</v>
       </c>
@@ -1053,140 +993,136 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="13" t="n">
+      <c r="B2" s="13">
         <v>11.3</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="n">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3">
         <v>2027</v>
       </c>
-      <c r="B3" s="13" t="n">
+      <c r="B3" s="13">
         <v>45.4</v>
       </c>
-      <c r="C3" s="12" t="n">
+      <c r="C3" s="12">
         <v>1162</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="n">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4">
         <v>2028</v>
       </c>
-      <c r="B4" s="13" t="n">
+      <c r="B4" s="13">
         <v>45</v>
       </c>
-      <c r="C4" s="12" t="n">
+      <c r="C4" s="12">
         <v>1085</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="n">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5">
         <v>2029</v>
       </c>
-      <c r="B5" s="13" t="n">
+      <c r="B5" s="13">
         <v>43.5</v>
       </c>
-      <c r="C5" s="12" t="n">
+      <c r="C5" s="12">
         <v>999</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="n">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6">
         <v>2030</v>
       </c>
-      <c r="B6" s="13" t="n">
+      <c r="B6" s="13">
         <v>40</v>
       </c>
-      <c r="C6" s="12" t="n">
+      <c r="C6" s="12">
         <v>909</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="n">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7">
         <v>2031</v>
       </c>
-      <c r="B7" s="13" t="n">
+      <c r="B7" s="13">
         <v>34.1</v>
       </c>
-      <c r="C7" s="12" t="n">
+      <c r="C7" s="12">
         <v>796</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="n">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8">
         <v>2032</v>
       </c>
-      <c r="B8" s="13" t="n">
+      <c r="B8" s="13">
         <v>29.4</v>
       </c>
-      <c r="C8" s="12" t="n">
+      <c r="C8" s="12">
         <v>669</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="n">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9">
         <v>2033</v>
       </c>
-      <c r="B9" s="13" t="n">
+      <c r="B9" s="13">
         <v>23.3</v>
       </c>
-      <c r="C9" s="12" t="n">
+      <c r="C9" s="12">
         <v>565</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="n">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10">
         <v>2034</v>
       </c>
-      <c r="B10" s="13" t="n">
+      <c r="B10" s="13">
         <v>16.9</v>
       </c>
-      <c r="C10" s="12" t="n">
+      <c r="C10" s="12">
         <v>381</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="n">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11">
         <v>2035</v>
       </c>
-      <c r="B11" s="13" t="n">
+      <c r="B11" s="13">
         <v>8.9</v>
       </c>
-      <c r="C11" s="12" t="n">
+      <c r="C11" s="12">
         <v>218</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="18" t="n">
+      <c r="B12" s="18">
         <v>297.9</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE4CD114-211B-4C53-A9CF-4B20BD64BEEF}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col min="1" max="1" width="30.7109375" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>21</v>
       </c>
@@ -1194,53 +1130,49 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>23</v>
       </c>
-      <c r="B2" s="13" t="n">
+      <c r="B2" s="13">
         <v>87.09999999999999</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="13" t="n">
+      <c r="B3" s="13">
         <v>121.7</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>25</v>
       </c>
-      <c r="B4" s="13" t="n">
+      <c r="B4" s="13">
         <v>89.09999999999999</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2806160-F711-43CF-8E1F-3F7BDB274815}">
   <dimension ref="A1:F7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col min="1" max="1" width="16.7109375" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" customWidth="1"/>
+    <col min="3" max="3" width="20.7109375" customWidth="1"/>
+    <col min="4" max="4" width="16.7109375" customWidth="1"/>
+    <col min="5" max="5" width="20.7109375" customWidth="1"/>
+    <col min="6" max="6" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>26</v>
       </c>
@@ -1260,165 +1192,161 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>32</v>
       </c>
-      <c r="B2" t="n">
+      <c r="B2">
         <v>5</v>
       </c>
-      <c r="C2" s="21" t="n">
+      <c r="C2" s="21">
         <v>2567.6</v>
       </c>
-      <c r="D2" s="22" t="n">
+      <c r="D2" s="22">
         <v>0.0019</v>
       </c>
-      <c r="E2" s="21" t="n">
+      <c r="E2" s="21">
         <v>2066</v>
       </c>
-      <c r="F2" s="13" t="n">
+      <c r="F2" s="13">
         <v>4</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>33</v>
       </c>
-      <c r="B3" t="n">
+      <c r="B3">
         <v>51</v>
       </c>
-      <c r="C3" s="21" t="n">
+      <c r="C3" s="21">
         <v>2228.3</v>
       </c>
-      <c r="D3" s="22" t="n">
+      <c r="D3" s="22">
         <v>0.0229</v>
       </c>
-      <c r="E3" s="21" t="n">
+      <c r="E3" s="21">
         <v>1187.1</v>
       </c>
-      <c r="F3" s="13" t="n">
+      <c r="F3" s="13">
         <v>27.2</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>34</v>
       </c>
-      <c r="B4" t="n">
+      <c r="B4">
         <v>61</v>
       </c>
-      <c r="C4" s="21" t="n">
+      <c r="C4" s="21">
         <v>1417.2</v>
       </c>
-      <c r="D4" s="22" t="n">
+      <c r="D4" s="22">
         <v>0.043</v>
       </c>
-      <c r="E4" s="21" t="n">
+      <c r="E4" s="21">
         <v>1838</v>
       </c>
-      <c r="F4" s="13" t="n">
+      <c r="F4" s="13">
         <v>79.09999999999999</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>35</v>
       </c>
-      <c r="B5" t="n">
+      <c r="B5">
         <v>66</v>
       </c>
-      <c r="C5" s="21" t="n">
+      <c r="C5" s="21">
         <v>662</v>
       </c>
-      <c r="D5" s="22" t="n">
+      <c r="D5" s="22">
         <v>0.0997</v>
       </c>
-      <c r="E5" s="21" t="n">
+      <c r="E5" s="21">
         <v>1141.5</v>
       </c>
-      <c r="F5" s="13" t="n">
+      <c r="F5" s="13">
         <v>113.8</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>36</v>
       </c>
-      <c r="B6" t="n">
+      <c r="B6">
         <v>14</v>
       </c>
-      <c r="C6" s="21" t="n">
+      <c r="C6" s="21">
         <v>56.5</v>
       </c>
-      <c r="D6" s="22" t="n">
+      <c r="D6" s="22">
         <v>0.2478</v>
       </c>
-      <c r="E6" s="21" t="n">
+      <c r="E6" s="21">
         <v>297.7</v>
       </c>
-      <c r="F6" s="13" t="n">
+      <c r="F6" s="13">
         <v>73.8</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B7" s="3" t="n">
+      <c r="B7" s="3">
         <v>197</v>
       </c>
-      <c r="F7" s="18" t="n">
+      <c r="F7" s="18">
         <v>297.9</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{962AD7E5-F2D7-450A-8E33-D77C76B13837}">
   <dimension ref="A1:A6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col width="120" customWidth="1" min="1" max="1"/>
+    <col min="1" max="1" width="120.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="23" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="23" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="23" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="23" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="23" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="23" t="s">
         <v>42</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
task132 realism repair 2: failure and stock tie-out, procedure definitions table, program scope off the register, crew text, a fuller extract, master data, RMA history, containers and Canadian spelling; answer still 13 lots, expected failures 298.9
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task132/golden/vpr340_psu_final_buy.xlsx
+++ b/task132/golden/vpr340_psu_final_buy.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27728"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E1A4429-1A48-47A3-B72C-345A18A5DECE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_{3E1A4429-1A48-47A3-B72C-345A18A5DECE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{AA6AA2A3-D398-41C7-A988-ABB893934BF3}"/>
   </bookViews>
@@ -133,7 +133,7 @@
     <t>25+</t>
   </si>
   <si>
-    <t>Failures: corrective (CM, EM) work orders on VPR-340 relays with failed component PSU, status COMP or CLOSE (AM-PC-014 5.1). Each failure takes the age of the module it removed, from that module's fitted date in the rotating-item history (5.2).</t>
+    <t>Failures: corrective (CM, EM) work orders on VPR-340 relays with failed component PSU, status COMP or CLOSE (AM-PC-014 5.1). Each failure takes the age of the module it removed, from that module's fitted date in the rotating-item history (5.2); legacy fitted dates held only as a year are used as loaded, 1 July of that year.</t>
   </si>
   <si>
     <t>Rates: module-years are counted from the January 2021 go-live, when the work-order history begins; a module fitted earlier enters the count at go-live at the age it had then (5.3).</t>
@@ -142,10 +142,10 @@
     <t>Expected module-years: each supported relay's present module is aged month by month. A module that fails is replaced from stock by a new module, which counts in the 0-9 band from the following month, so each month's module-years are split between the present module (by the chance it has not yet failed) and its replacement (6.1, 6.2).</t>
   </si>
   <si>
-    <t>Support ends in the commissioning month of the scheme, or the stage of a staged scheme, that replaces the relay's bay in the approved 2026 programme; relays at stations with no scheme in the period are supported to December 2035 (4.1, 4.2).</t>
-  </si>
-  <si>
-    <t>Available modules: 12 serviceable at Central Stores, North and South depots plus 2 at Veldtek under open RMA; 7 quarantined modules excluded (7).</t>
+    <t>Support ends in the commissioning month of the scheme, or the stage of a staged scheme, that replaces the relay's bay in the approved 2026 program; relays at stations with no scheme in the period are supported to December 2035 (4.1, 4.2).</t>
+  </si>
+  <si>
+    <t>Available modules: 12 serviceable at Central Stores, North and South depots plus 3 at Veldtek under open RMA; 7 quarantined modules excluded (7).</t>
   </si>
   <si>
     <t>Cover is the Poisson probability that available modules plus the buy meet all failures to end of support (8.1, 8.2).</t>
@@ -610,7 +610,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="7">
-        <v>297.9</v>
+        <v>298.9</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -618,7 +618,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="8">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -675,7 +675,7 @@
         <v>200</v>
       </c>
       <c r="C2" s="12">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D2" s="13">
         <v>0</v>
@@ -695,7 +695,7 @@
         <v>225</v>
       </c>
       <c r="C3" s="12">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D3" s="13">
         <v>0</v>
@@ -715,7 +715,7 @@
         <v>250</v>
       </c>
       <c r="C4" s="12">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D4" s="13">
         <v>2.5</v>
@@ -735,7 +735,7 @@
         <v>275</v>
       </c>
       <c r="C5" s="12">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D5" s="13">
         <v>31.6</v>
@@ -755,7 +755,7 @@
         <v>300</v>
       </c>
       <c r="C6" s="12">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="D6" s="13">
         <v>83.2</v>
@@ -775,7 +775,7 @@
         <v>325</v>
       </c>
       <c r="C7" s="17">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="D7" s="18">
         <v>99.09999999999999</v>
@@ -795,7 +795,7 @@
         <v>350</v>
       </c>
       <c r="C8" s="12">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="D8" s="13">
         <v>100</v>
@@ -815,7 +815,7 @@
         <v>375</v>
       </c>
       <c r="C9" s="12">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="D9" s="13">
         <v>100</v>
@@ -835,7 +835,7 @@
         <v>400</v>
       </c>
       <c r="C10" s="12">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="D10" s="13">
         <v>100</v>
@@ -855,7 +855,7 @@
         <v>425</v>
       </c>
       <c r="C11" s="12">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="D11" s="13">
         <v>100</v>
@@ -875,7 +875,7 @@
         <v>450</v>
       </c>
       <c r="C12" s="12">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="D12" s="13">
         <v>100</v>
@@ -895,7 +895,7 @@
         <v>475</v>
       </c>
       <c r="C13" s="12">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="D13" s="13">
         <v>100</v>
@@ -915,7 +915,7 @@
         <v>500</v>
       </c>
       <c r="C14" s="12">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="D14" s="13">
         <v>100</v>
@@ -935,7 +935,7 @@
         <v>525</v>
       </c>
       <c r="C15" s="12">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="D15" s="13">
         <v>100</v>
@@ -955,7 +955,7 @@
         <v>550</v>
       </c>
       <c r="C16" s="12">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D16" s="13">
         <v>100</v>
@@ -998,7 +998,7 @@
         <v>19</v>
       </c>
       <c r="B2" s="13">
-        <v>11.3</v>
+        <v>11.4</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -1006,7 +1006,7 @@
         <v>2027</v>
       </c>
       <c r="B3" s="13">
-        <v>45.4</v>
+        <v>45.6</v>
       </c>
       <c r="C3" s="12">
         <v>1162</v>
@@ -1017,7 +1017,7 @@
         <v>2028</v>
       </c>
       <c r="B4" s="13">
-        <v>45</v>
+        <v>45.2</v>
       </c>
       <c r="C4" s="12">
         <v>1085</v>
@@ -1028,7 +1028,7 @@
         <v>2029</v>
       </c>
       <c r="B5" s="13">
-        <v>43.5</v>
+        <v>43.7</v>
       </c>
       <c r="C5" s="12">
         <v>999</v>
@@ -1039,7 +1039,7 @@
         <v>2030</v>
       </c>
       <c r="B6" s="13">
-        <v>40</v>
+        <v>40.1</v>
       </c>
       <c r="C6" s="12">
         <v>909</v>
@@ -1050,7 +1050,7 @@
         <v>2031</v>
       </c>
       <c r="B7" s="13">
-        <v>34.1</v>
+        <v>34.2</v>
       </c>
       <c r="C7" s="12">
         <v>796</v>
@@ -1083,7 +1083,7 @@
         <v>2034</v>
       </c>
       <c r="B10" s="13">
-        <v>16.9</v>
+        <v>17</v>
       </c>
       <c r="C10" s="12">
         <v>381</v>
@@ -1105,7 +1105,7 @@
         <v>20</v>
       </c>
       <c r="B12" s="18">
-        <v>297.9</v>
+        <v>298.9</v>
       </c>
     </row>
   </sheetData>
@@ -1135,7 +1135,7 @@
         <v>23</v>
       </c>
       <c r="B2" s="13">
-        <v>87.09999999999999</v>
+        <v>87.2</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1143,7 +1143,7 @@
         <v>24</v>
       </c>
       <c r="B3" s="13">
-        <v>121.7</v>
+        <v>122.1</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1151,7 +1151,7 @@
         <v>25</v>
       </c>
       <c r="B4" s="13">
-        <v>89.09999999999999</v>
+        <v>89.59999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -1206,7 +1206,7 @@
         <v>0.0019</v>
       </c>
       <c r="E2" s="21">
-        <v>2066</v>
+        <v>2068.8</v>
       </c>
       <c r="F2" s="13">
         <v>4</v>
@@ -1220,13 +1220,13 @@
         <v>51</v>
       </c>
       <c r="C3" s="21">
-        <v>2228.3</v>
+        <v>2228.2</v>
       </c>
       <c r="D3" s="22">
         <v>0.0229</v>
       </c>
       <c r="E3" s="21">
-        <v>1187.1</v>
+        <v>1187.2</v>
       </c>
       <c r="F3" s="13">
         <v>27.2</v>
@@ -1240,13 +1240,13 @@
         <v>61</v>
       </c>
       <c r="C4" s="21">
-        <v>1417.2</v>
+        <v>1417.3</v>
       </c>
       <c r="D4" s="22">
         <v>0.043</v>
       </c>
       <c r="E4" s="21">
-        <v>1838</v>
+        <v>1837.7</v>
       </c>
       <c r="F4" s="13">
         <v>79.09999999999999</v>
@@ -1260,16 +1260,16 @@
         <v>66</v>
       </c>
       <c r="C5" s="21">
-        <v>662</v>
+        <v>663.5</v>
       </c>
       <c r="D5" s="22">
-        <v>0.0997</v>
+        <v>0.09950000000000001</v>
       </c>
       <c r="E5" s="21">
-        <v>1141.5</v>
+        <v>1142</v>
       </c>
       <c r="F5" s="13">
-        <v>113.8</v>
+        <v>113.6</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -1280,16 +1280,16 @@
         <v>14</v>
       </c>
       <c r="C6" s="21">
-        <v>56.5</v>
+        <v>55</v>
       </c>
       <c r="D6" s="22">
-        <v>0.2478</v>
+        <v>0.2545</v>
       </c>
       <c r="E6" s="21">
-        <v>297.7</v>
+        <v>294.7</v>
       </c>
       <c r="F6" s="13">
-        <v>73.8</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -1300,7 +1300,7 @@
         <v>197</v>
       </c>
       <c r="F7" s="18">
-        <v>297.9</v>
+        <v>298.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
task132 realism repair 3: exposure window and end of support pinned, early-life and random failures with warranty returns, rebuild modules scrapped under e-waste manifests, procedure history from first issue, crew text, EAM residue, late-2026 commissionings, LibreOffice EOL notice, fixed-decimal CSVs and Excel caches; answer still 13 lots (298.6 expected failures), no-renewal stump 19 lots
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task132/golden/vpr340_psu_final_buy.xlsx
+++ b/task132/golden/vpr340_psu_final_buy.xlsx
@@ -142,7 +142,7 @@
     <t>Expected module-years: each supported relay's present module is aged month by month. A module that fails is replaced from stock by a new module, which counts in the 0-9 band from the following month, so each month's module-years are split between the present module (by the chance it has not yet failed) and its replacement (6.1, 6.2).</t>
   </si>
   <si>
-    <t>Support ends in the commissioning month of the scheme, or the stage of a staged scheme, that replaces the relay's bay in the approved 2026 program; relays at stations with no scheme in the period are supported to December 2035 (4.1, 4.2).</t>
+    <t>Support ends in the commissioning month of the scheme, or the stage of a staged scheme, that replaces the relay's bay in the approved 2026 program; relays at stations with no scheme in the period are supported through December 2035 (4.1, 4.2).</t>
   </si>
   <si>
     <t>Available modules: 12 serviceable at Central Stores, North and South depots plus 3 at Veldtek under open RMA; 7 quarantined modules excluded (7).</t>
@@ -610,7 +610,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="7">
-        <v>298.9</v>
+        <v>298.6</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -626,7 +626,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="9">
-        <v>99.09999999999999</v>
+        <v>99.1</v>
       </c>
     </row>
   </sheetData>
@@ -718,7 +718,7 @@
         <v>265</v>
       </c>
       <c r="D4" s="13">
-        <v>2.5</v>
+        <v>2.6</v>
       </c>
       <c r="E4" s="14">
         <v>491250</v>
@@ -738,7 +738,7 @@
         <v>290</v>
       </c>
       <c r="D5" s="13">
-        <v>31.6</v>
+        <v>32.2</v>
       </c>
       <c r="E5" s="14">
         <v>540375</v>
@@ -758,7 +758,7 @@
         <v>315</v>
       </c>
       <c r="D6" s="13">
-        <v>83.2</v>
+        <v>83.6</v>
       </c>
       <c r="E6" s="14">
         <v>589500</v>
@@ -778,7 +778,7 @@
         <v>340</v>
       </c>
       <c r="D7" s="18">
-        <v>99.09999999999999</v>
+        <v>99.1</v>
       </c>
       <c r="E7" s="19">
         <v>638625</v>
@@ -998,7 +998,7 @@
         <v>19</v>
       </c>
       <c r="B2" s="13">
-        <v>11.4</v>
+        <v>11.6</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -1006,10 +1006,10 @@
         <v>2027</v>
       </c>
       <c r="B3" s="13">
-        <v>45.6</v>
+        <v>45.1</v>
       </c>
       <c r="C3" s="12">
-        <v>1162</v>
+        <v>1163</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -1017,10 +1017,10 @@
         <v>2028</v>
       </c>
       <c r="B4" s="13">
-        <v>45.2</v>
+        <v>44.7</v>
       </c>
       <c r="C4" s="12">
-        <v>1085</v>
+        <v>1094</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -1028,10 +1028,10 @@
         <v>2029</v>
       </c>
       <c r="B5" s="13">
-        <v>43.7</v>
+        <v>42.9</v>
       </c>
       <c r="C5" s="12">
-        <v>999</v>
+        <v>973</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -1039,10 +1039,10 @@
         <v>2030</v>
       </c>
       <c r="B6" s="13">
-        <v>40.1</v>
+        <v>40.6</v>
       </c>
       <c r="C6" s="12">
-        <v>909</v>
+        <v>884</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -1050,10 +1050,10 @@
         <v>2031</v>
       </c>
       <c r="B7" s="13">
-        <v>34.2</v>
+        <v>36.1</v>
       </c>
       <c r="C7" s="12">
-        <v>796</v>
+        <v>783</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -1061,10 +1061,10 @@
         <v>2032</v>
       </c>
       <c r="B8" s="13">
-        <v>29.4</v>
+        <v>30</v>
       </c>
       <c r="C8" s="12">
-        <v>669</v>
+        <v>695</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -1072,10 +1072,10 @@
         <v>2033</v>
       </c>
       <c r="B9" s="13">
-        <v>23.3</v>
+        <v>23.9</v>
       </c>
       <c r="C9" s="12">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -1083,10 +1083,10 @@
         <v>2034</v>
       </c>
       <c r="B10" s="13">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C10" s="12">
-        <v>381</v>
+        <v>373</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -1094,10 +1094,10 @@
         <v>2035</v>
       </c>
       <c r="B11" s="13">
-        <v>8.9</v>
+        <v>7.8</v>
       </c>
       <c r="C11" s="12">
-        <v>218</v>
+        <v>201</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -1105,7 +1105,7 @@
         <v>20</v>
       </c>
       <c r="B12" s="18">
-        <v>298.9</v>
+        <v>298.6</v>
       </c>
     </row>
   </sheetData>
@@ -1135,7 +1135,7 @@
         <v>23</v>
       </c>
       <c r="B2" s="13">
-        <v>87.2</v>
+        <v>117.5</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1143,7 +1143,7 @@
         <v>24</v>
       </c>
       <c r="B3" s="13">
-        <v>122.1</v>
+        <v>54.7</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1151,7 +1151,7 @@
         <v>25</v>
       </c>
       <c r="B4" s="13">
-        <v>89.59999999999999</v>
+        <v>126.4</v>
       </c>
     </row>
   </sheetData>
@@ -1197,19 +1197,19 @@
         <v>32</v>
       </c>
       <c r="B2">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="C2" s="21">
-        <v>2567.6</v>
+        <v>2905.8</v>
       </c>
       <c r="D2" s="22">
-        <v>0.0019</v>
+        <v>0.0052</v>
       </c>
       <c r="E2" s="21">
-        <v>2068.8</v>
+        <v>2206.2</v>
       </c>
       <c r="F2" s="13">
-        <v>4</v>
+        <v>11.4</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -1217,19 +1217,19 @@
         <v>33</v>
       </c>
       <c r="B3">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C3" s="21">
-        <v>2228.2</v>
+        <v>2104.4</v>
       </c>
       <c r="D3" s="22">
-        <v>0.0229</v>
+        <v>0.0233</v>
       </c>
       <c r="E3" s="21">
-        <v>1187.2</v>
+        <v>1466.2</v>
       </c>
       <c r="F3" s="13">
-        <v>27.2</v>
+        <v>34.1</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -1237,19 +1237,19 @@
         <v>34</v>
       </c>
       <c r="B4">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="C4" s="21">
-        <v>1417.3</v>
+        <v>1337.4</v>
       </c>
       <c r="D4" s="22">
-        <v>0.043</v>
+        <v>0.0508</v>
       </c>
       <c r="E4" s="21">
-        <v>1837.7</v>
+        <v>1704.6</v>
       </c>
       <c r="F4" s="13">
-        <v>79.09999999999999</v>
+        <v>86.7</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -1260,16 +1260,16 @@
         <v>66</v>
       </c>
       <c r="C5" s="21">
-        <v>663.5</v>
+        <v>556.3</v>
       </c>
       <c r="D5" s="22">
-        <v>0.09950000000000001</v>
+        <v>0.1186</v>
       </c>
       <c r="E5" s="21">
-        <v>1142</v>
+        <v>868.9</v>
       </c>
       <c r="F5" s="13">
-        <v>113.6</v>
+        <v>103.1</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -1277,19 +1277,19 @@
         <v>36</v>
       </c>
       <c r="B6">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C6" s="21">
-        <v>55</v>
+        <v>40.8</v>
       </c>
       <c r="D6" s="22">
-        <v>0.2545</v>
+        <v>0.2945</v>
       </c>
       <c r="E6" s="21">
-        <v>294.7</v>
+        <v>215.1</v>
       </c>
       <c r="F6" s="13">
-        <v>75</v>
+        <v>63.3</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -1297,10 +1297,10 @@
         <v>20</v>
       </c>
       <c r="B7" s="3">
-        <v>197</v>
+        <v>210</v>
       </c>
       <c r="F7" s="18">
-        <v>298.9</v>
+        <v>298.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>